<commit_message>
Minor changes and additional sensitivity analyses
</commit_message>
<xml_diff>
--- a/detection_mode_project/outputs/sensitivity_results_gsvar.xlsx
+++ b/detection_mode_project/outputs/sensitivity_results_gsvar.xlsx
@@ -363,13 +363,13 @@
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>**Interval**  
-N = 509</t>
+N = 534</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
           <t>**Screen-Detected**  
-N = 827</t>
+N = 852</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -448,12 +448,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>103 (20)</t>
+          <t>110 (21)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>197 (24)</t>
+          <t>200 (23)</t>
         </is>
       </c>
     </row>
@@ -465,72 +465,72 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>251 (49)</t>
+          <t>262 (49)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>372 (45)</t>
+          <t>384 (45)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.30</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.95, 1.79</t>
+          <t>0.91, 1.69</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.103</t>
+          <t>0.170</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>1.28</t>
+          <t>1.22</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0.92, 1.78</t>
+          <t>0.88, 1.67</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0.146</t>
+          <t>0.231</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>1.38</t>
+          <t>1.35</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>0.97, 1.97</t>
+          <t>0.96, 1.91</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0.073</t>
+          <t>0.090</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.90, 1.87</t>
+          <t>0.89, 1.80</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0.166</t>
+          <t>0.199</t>
         </is>
       </c>
     </row>
@@ -542,72 +542,72 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>109 (21)</t>
+          <t>114 (21)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>190 (23)</t>
+          <t>195 (23)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>0.98</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.70, 1.47</t>
+          <t>0.68, 1.40</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.943</t>
+          <t>0.904</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0.98</t>
+          <t>0.94</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0.67, 1.45</t>
+          <t>0.65, 1.37</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0.923</t>
+          <t>0.755</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>1.08</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>0.72, 1.65</t>
+          <t>0.72, 1.62</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0.680</t>
+          <t>0.703</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>0.66, 1.54</t>
+          <t>0.66, 1.51</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>0.978</t>
+          <t>0.992</t>
         </is>
       </c>
     </row>
@@ -619,12 +619,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>46 (9.0)</t>
+          <t>48 (9.0)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>68 (8.2)</t>
+          <t>73 (8.6)</t>
         </is>
       </c>
     </row>
@@ -643,12 +643,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>64 (13)</t>
+          <t>70 (13)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>140 (17)</t>
+          <t>144 (17)</t>
         </is>
       </c>
     </row>
@@ -660,72 +660,72 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>444 (87)</t>
+          <t>463 (87)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>685 (83)</t>
+          <t>706 (83)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.84, 1.75</t>
+          <t>0.81, 1.65</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0.315</t>
+          <t>0.421</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0.85, 1.82</t>
+          <t>0.82, 1.70</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>0.268</t>
+          <t>0.380</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>1.22</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>0.82, 1.83</t>
+          <t>0.81, 1.77</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0.328</t>
+          <t>0.369</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>0.82, 1.88</t>
+          <t>0.81, 1.81</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>0.323</t>
+          <t>0.370</t>
         </is>
       </c>
     </row>
@@ -761,12 +761,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>59 (12)</t>
+          <t>62 (12)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>108 (13)</t>
+          <t>110 (13)</t>
         </is>
       </c>
     </row>
@@ -778,72 +778,72 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>56 (11)</t>
+          <t>60 (11)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>86 (10)</t>
+          <t>90 (11)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1.72</t>
+          <t>1.60</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.76, 3.90</t>
+          <t>0.72, 3.56</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.191</t>
+          <t>0.248</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>1.87</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>0.80, 4.37</t>
+          <t>0.75, 3.97</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>0.149</t>
+          <t>0.198</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>1.53</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>0.63, 3.73</t>
+          <t>0.54, 3.10</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0.347</t>
+          <t>0.567</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>1.58</t>
+          <t>1.35</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>0.63, 3.95</t>
+          <t>0.55, 3.33</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>0.331</t>
+          <t>0.511</t>
         </is>
       </c>
     </row>
@@ -855,72 +855,72 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>279 (55)</t>
+          <t>290 (54)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>443 (54)</t>
+          <t>458 (54)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.38</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0.74, 3.18</t>
+          <t>0.67, 2.82</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.248</t>
+          <t>0.377</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>0.75, 3.47</t>
+          <t>0.68, 3.08</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>0.220</t>
+          <t>0.333</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>1.20</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>0.54, 2.65</t>
+          <t>0.45, 2.19</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0.649</t>
+          <t>0.998</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>1.05</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>0.54, 2.78</t>
+          <t>0.46, 2.34</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>0.624</t>
+          <t>0.914</t>
         </is>
       </c>
     </row>
@@ -932,72 +932,72 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>115 (23)</t>
+          <t>122 (23)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>190 (23)</t>
+          <t>194 (23)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0.62, 2.80</t>
+          <t>0.60, 2.64</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.464</t>
+          <t>0.532</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>1.38</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>0.62, 3.04</t>
+          <t>0.62, 2.92</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>0.423</t>
+          <t>0.455</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.03</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>0.51, 2.62</t>
+          <t>0.46, 2.31</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0.718</t>
+          <t>0.939</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.08</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>0.50, 2.71</t>
+          <t>0.46, 2.48</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>0.724</t>
+          <t>0.860</t>
         </is>
       </c>
     </row>
@@ -1016,12 +1016,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>26 (5.1)</t>
+          <t>26 (4.9)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>31 (3.7)</t>
+          <t>32 (3.8)</t>
         </is>
       </c>
     </row>
@@ -1033,72 +1033,72 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>135 (27)</t>
+          <t>142 (27)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>229 (28)</t>
+          <t>236 (28)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.71</t>
+          <t>0.77</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0.38, 1.33</t>
+          <t>0.42, 1.42</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0.286</t>
+          <t>0.396</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0.73</t>
+          <t>0.76</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>0.38, 1.42</t>
+          <t>0.40, 1.47</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>0.348</t>
+          <t>0.417</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>0.68</t>
+          <t>0.76</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>0.34, 1.34</t>
+          <t>0.39, 1.50</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0.259</t>
+          <t>0.424</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>0.71</t>
+          <t>0.77</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>0.35, 1.44</t>
+          <t>0.39, 1.55</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.342</t>
+          <t>0.456</t>
         </is>
       </c>
     </row>
@@ -1110,72 +1110,72 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>183 (36)</t>
+          <t>192 (36)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>299 (36)</t>
+          <t>305 (36)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.68</t>
+          <t>0.76</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0.36, 1.27</t>
+          <t>0.41, 1.41</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0.219</t>
+          <t>0.382</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>0.68</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>0.36, 1.32</t>
+          <t>0.39, 1.43</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>0.250</t>
+          <t>0.372</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>0.68</t>
+          <t>0.81</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>0.35, 1.35</t>
+          <t>0.42, 1.59</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0.271</t>
+          <t>0.541</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>0.82</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>0.36, 1.45</t>
+          <t>0.41, 1.64</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>0.350</t>
+          <t>0.567</t>
         </is>
       </c>
     </row>
@@ -1187,72 +1187,72 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>78 (15)</t>
+          <t>83 (16)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>113 (14)</t>
+          <t>120 (14)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.68</t>
+          <t>0.76</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>0.35, 1.35</t>
+          <t>0.39, 1.49</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0.272</t>
+          <t>0.426</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>0.71</t>
+          <t>0.78</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>0.35, 1.45</t>
+          <t>0.39, 1.57</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>0.344</t>
+          <t>0.479</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>0.67</t>
+          <t>0.81</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>0.32, 1.42</t>
+          <t>0.39, 1.68</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0.297</t>
+          <t>0.561</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>0.71</t>
+          <t>0.82</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>0.33, 1.53</t>
+          <t>0.39, 1.74</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>0.378</t>
+          <t>0.600</t>
         </is>
       </c>
     </row>
@@ -1264,72 +1264,72 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>26 (5.1)</t>
+          <t>27 (5.1)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>42 (5.1)</t>
+          <t>44 (5.2)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0.63</t>
+          <t>0.69</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>0.27, 1.43</t>
+          <t>0.31, 1.56</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0.266</t>
+          <t>0.377</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>0.73</t>
+          <t>0.79</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0.31, 1.70</t>
+          <t>0.34, 1.81</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>0.464</t>
+          <t>0.574</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>0.66</t>
+          <t>0.76</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>0.27, 1.62</t>
+          <t>0.31, 1.84</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0.361</t>
+          <t>0.541</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.83</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>0.30, 1.88</t>
+          <t>0.34, 2.05</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>0.531</t>
+          <t>0.681</t>
         </is>
       </c>
     </row>
@@ -1341,12 +1341,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>61 (12)</t>
+          <t>64 (12)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>113 (14)</t>
+          <t>115 (13)</t>
         </is>
       </c>
     </row>
@@ -1365,12 +1365,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>69 (14)</t>
+          <t>73 (14)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>135 (16)</t>
+          <t>140 (16)</t>
         </is>
       </c>
     </row>
@@ -1382,72 +1382,72 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>140 (28)</t>
+          <t>150 (28)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>238 (29)</t>
+          <t>244 (29)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1.22</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>0.82, 1.81</t>
+          <t>0.85, 1.82</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0.323</t>
+          <t>0.272</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>0.82, 1.87</t>
+          <t>0.85, 1.88</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>0.309</t>
+          <t>0.253</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>1.30</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>0.84, 2.00</t>
+          <t>0.87, 2.02</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0.241</t>
+          <t>0.195</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>1.31</t>
+          <t>1.33</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>0.83, 2.06</t>
+          <t>0.86, 2.07</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>0.246</t>
+          <t>0.199</t>
         </is>
       </c>
     </row>
@@ -1459,72 +1459,72 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>98 (19)</t>
+          <t>101 (19)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>136 (16)</t>
+          <t>140 (16)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1.30</t>
+          <t>1.23</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0.85, 2.01</t>
+          <t>0.81, 1.88</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>0.230</t>
+          <t>0.334</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.23</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>0.82, 2.02</t>
+          <t>0.80, 1.90</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>0.272</t>
+          <t>0.352</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>1.53</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>0.95, 2.46</t>
+          <t>0.91, 2.32</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0.082</t>
+          <t>0.116</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>1.52</t>
+          <t>1.47</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>0.93, 2.50</t>
+          <t>0.91, 2.38</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>0.099</t>
+          <t>0.118</t>
         </is>
       </c>
     </row>
@@ -1536,72 +1536,72 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>93 (18)</t>
+          <t>96 (18)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>163 (20)</t>
+          <t>169 (20)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>1.08</t>
+          <t>1.04</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>0.69, 1.68</t>
+          <t>0.67, 1.60</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>0.744</t>
+          <t>0.869</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>0.99</t>
+          <t>0.95</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>0.62, 1.58</t>
+          <t>0.61, 1.48</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>0.968</t>
+          <t>0.807</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>0.75, 1.98</t>
+          <t>0.70, 1.81</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0.438</t>
+          <t>0.630</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.03</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>0.68, 1.88</t>
+          <t>0.63, 1.69</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>0.629</t>
+          <t>0.895</t>
         </is>
       </c>
     </row>
@@ -1613,72 +1613,72 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>50 (9.8)</t>
+          <t>52 (9.7)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>47 (5.7)</t>
+          <t>49 (5.8)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>1.95</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.20, 3.75</t>
+          <t>1.12, 3.40</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0.010</t>
+          <t>0.019</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>1.96</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1.17, 3.82</t>
+          <t>1.11, 3.49</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>0.013</t>
+          <t>0.021</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2.43</t>
+          <t>2.32</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>1.31, 4.52</t>
+          <t>1.27, 4.26</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0.005</t>
+          <t>0.006</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>2.38</t>
+          <t>2.28</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>1.26, 4.54</t>
+          <t>1.23, 4.27</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>0.008</t>
+          <t>0.009</t>
         </is>
       </c>
     </row>
@@ -1690,12 +1690,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>59 (12)</t>
+          <t>62 (12)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>108 (13)</t>
+          <t>110 (13)</t>
         </is>
       </c>
     </row>
@@ -1714,12 +1714,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>156 (31)</t>
+          <t>159 (30)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>200 (24)</t>
+          <t>207 (24)</t>
         </is>
       </c>
     </row>
@@ -1731,72 +1731,72 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>353 (69)</t>
+          <t>375 (70)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>627 (76)</t>
+          <t>645 (76)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0.63</t>
+          <t>0.66</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>0.38, 1.03</t>
+          <t>0.41, 1.06</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>0.065</t>
+          <t>0.085</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>0.43, 1.21</t>
+          <t>0.45, 1.23</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>0.221</t>
+          <t>0.250</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>0.68</t>
+          <t>0.71</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>0.39, 1.17</t>
+          <t>0.41, 1.20</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0.169</t>
+          <t>0.201</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>0.77</t>
+          <t>0.79</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>0.43, 1.35</t>
+          <t>0.46, 1.37</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>0.361</t>
+          <t>0.403</t>
         </is>
       </c>
     </row>
@@ -1815,12 +1815,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>69 (14)</t>
+          <t>78 (15)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>143 (17)</t>
+          <t>147 (17)</t>
         </is>
       </c>
     </row>
@@ -1832,72 +1832,72 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>238 (47)</t>
+          <t>246 (46)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>424 (51)</t>
+          <t>436 (51)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>0.97</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>0.78, 1.59</t>
+          <t>0.69, 1.37</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>0.571</t>
+          <t>0.866</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>0.71, 1.45</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>0.935</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>0.77, 1.64</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>0.562</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
           <t>1.16</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>0.80, 1.69</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>0.442</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>1.23</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>0.83, 1.83</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>0.302</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>1.27</t>
-        </is>
-      </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>0.85, 1.92</t>
+          <t>0.79, 1.73</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>0.248</t>
+          <t>0.446</t>
         </is>
       </c>
     </row>
@@ -1909,72 +1909,72 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>45 (8.8)</t>
+          <t>50 (9.4)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>56 (6.8)</t>
+          <t>58 (6.8)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>1.97</t>
+          <t>1.80</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.14, 3.40</t>
+          <t>1.07, 3.04</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>0.015</t>
+          <t>0.027</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>1.93</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1.19, 3.70</t>
+          <t>1.13, 3.31</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>0.010</t>
+          <t>0.016</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2.09</t>
+          <t>2.02</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>1.14, 3.82</t>
+          <t>1.14, 3.59</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0.017</t>
+          <t>0.016</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>2.15</t>
+          <t>2.12</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>1.15, 4.03</t>
+          <t>1.17, 3.85</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>0.017</t>
+          <t>0.013</t>
         </is>
       </c>
     </row>
@@ -1986,12 +1986,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>157 (31)</t>
+          <t>160 (30)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>204 (25)</t>
+          <t>211 (25)</t>
         </is>
       </c>
     </row>
@@ -2010,12 +2010,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>133 (26)</t>
+          <t>142 (27)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>254 (31)</t>
+          <t>267 (31)</t>
         </is>
       </c>
     </row>
@@ -2027,72 +2027,72 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>107 (21)</t>
+          <t>112 (21)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>223 (27)</t>
+          <t>229 (27)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
+          <t>0.92</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>0.66, 1.29</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>0.636</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>0.89</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>0.63, 1.27</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>0.523</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
           <t>0.95</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>0.67, 1.35</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>0.793</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>0.93</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>0.65, 1.34</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>0.708</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>1.00</t>
-        </is>
-      </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>0.68, 1.47</t>
+          <t>0.66, 1.38</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>0.993</t>
+          <t>0.800</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>0.98</t>
+          <t>0.92</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>0.66, 1.46</t>
+          <t>0.62, 1.35</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>0.925</t>
+          <t>0.672</t>
         </is>
       </c>
     </row>
@@ -2104,72 +2104,72 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>112 (22)</t>
+          <t>119 (22)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>147 (18)</t>
+          <t>146 (17)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>1.52</t>
+          <t>1.62</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>1.06, 2.19</t>
+          <t>1.14, 2.31</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>0.024</t>
+          <t>0.008</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>0.91, 1.95</t>
+          <t>1.00, 2.08</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>0.134</t>
+          <t>0.051</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>1.62</t>
+          <t>1.67</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>1.09, 2.42</t>
+          <t>1.13, 2.47</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>0.018</t>
+          <t>0.011</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>1.43</t>
+          <t>1.48</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>0.94, 2.17</t>
+          <t>0.99, 2.22</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>0.094</t>
+          <t>0.058</t>
         </is>
       </c>
     </row>
@@ -2181,12 +2181,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>157 (31)</t>
+          <t>161 (30)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>203 (25)</t>
+          <t>210 (25)</t>
         </is>
       </c>
     </row>
@@ -2205,12 +2205,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>309 (61)</t>
+          <t>323 (60)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>586 (71)</t>
+          <t>601 (71)</t>
         </is>
       </c>
     </row>
@@ -2222,22 +2222,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>200 (39)</t>
+          <t>211 (40)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>241 (29)</t>
+          <t>251 (29)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>1.67</t>
+          <t>1.64</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.29, 2.15</t>
+          <t>1.28, 2.10</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2247,12 +2247,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>1.48</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>1.15, 1.95</t>
+          <t>1.14, 1.91</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2262,12 +2262,12 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>1.84</t>
+          <t>1.80</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>1.39, 2.44</t>
+          <t>1.37, 2.36</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -2277,17 +2277,17 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>1.64</t>
+          <t>1.61</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>1.23, 2.21</t>
+          <t>1.21, 2.15</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>&lt;0.001</t>
+          <t>0.001</t>
         </is>
       </c>
     </row>
@@ -2306,12 +2306,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>378 (74)</t>
+          <t>401 (75)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>649 (78)</t>
+          <t>670 (79)</t>
         </is>
       </c>
     </row>
@@ -2323,72 +2323,72 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>131 (26)</t>
+          <t>133 (25)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>178 (22)</t>
+          <t>182 (21)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>1.01, 1.78</t>
+          <t>0.94, 1.64</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>0.044</t>
+          <t>0.126</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>1.35</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>1.00, 1.81</t>
+          <t>0.93, 1.66</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>0.046</t>
+          <t>0.133</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>1.53</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>1.12, 2.10</t>
+          <t>1.03, 1.92</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>0.007</t>
+          <t>0.029</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>1.53</t>
+          <t>1.40</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>1.11, 2.12</t>
+          <t>1.02, 1.92</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>0.010</t>
+          <t>0.038</t>
         </is>
       </c>
     </row>
@@ -2417,62 +2417,62 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2.08</t>
+          <t>1.88</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>0.31, 17.0</t>
+          <t>0.29, 15.1</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>0.445</t>
+          <t>0.508</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>3.06</t>
+          <t>2.64</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>0.43, 26.6</t>
+          <t>0.38, 22.2</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>0.264</t>
+          <t>0.322</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2.00</t>
+          <t>2.02</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>0.27, 18.7</t>
+          <t>0.27, 18.8</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>0.506</t>
+          <t>0.496</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>2.80</t>
+          <t>2.71</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>0.36, 27.4</t>
+          <t>0.36, 26.0</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>0.330</t>
+          <t>0.339</t>
         </is>
       </c>
     </row>
@@ -2484,12 +2484,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>289 (57)</t>
+          <t>301 (56)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>374 (45)</t>
+          <t>383 (45)</t>
         </is>
       </c>
     </row>
@@ -2501,22 +2501,22 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>138 (27)</t>
+          <t>146 (27)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>283 (34)</t>
+          <t>293 (34)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>0.68</t>
+          <t>0.69</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>0.51, 0.90</t>
+          <t>0.52, 0.90</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2531,22 +2531,22 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>0.59, 1.07</t>
+          <t>0.59, 1.05</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>0.125</t>
+          <t>0.102</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>0.66</t>
+          <t>0.67</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>0.48, 0.90</t>
+          <t>0.49, 0.90</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
@@ -2556,17 +2556,17 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>0.80</t>
+          <t>0.78</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>0.57, 1.10</t>
+          <t>0.56, 1.07</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>0.173</t>
+          <t>0.119</t>
         </is>
       </c>
     </row>
@@ -2578,72 +2578,72 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>72 (14)</t>
+          <t>77 (14)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>159 (19)</t>
+          <t>165 (19)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>0.65</t>
+          <t>0.66</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>0.45, 0.93</t>
+          <t>0.46, 0.94</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>0.019</t>
+          <t>0.021</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>0.84</t>
+          <t>0.82</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>0.56, 1.24</t>
+          <t>0.56, 1.19</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>0.373</t>
+          <t>0.290</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>0.57</t>
+          <t>0.59</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>0.38, 0.85</t>
+          <t>0.40, 0.88</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>0.007</t>
+          <t>0.009</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.74</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>0.49, 1.16</t>
+          <t>0.49, 1.12</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>0.197</t>
+          <t>0.161</t>
         </is>
       </c>
     </row>
@@ -2655,7 +2655,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>7 (1.4)</t>
+          <t>7 (1.3)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2679,72 +2679,72 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>49 (9.6)</t>
+          <t>52 (9.7)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>47 (5.7)</t>
+          <t>48 (5.6)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>1.55</t>
+          <t>1.62</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>0.96, 2.50</t>
+          <t>1.02, 2.58</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>0.071</t>
+          <t>0.039</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.79</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1.06, 2.83</t>
+          <t>1.12, 2.89</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>0.029</t>
+          <t>0.016</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>1.59</t>
+          <t>1.61</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>0.94, 2.69</t>
+          <t>0.97, 2.69</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>0.082</t>
+          <t>0.068</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>1.70</t>
+          <t>1.71</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>0.99, 2.93</t>
+          <t>1.01, 2.90</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>0.056</t>
+          <t>0.046</t>
         </is>
       </c>
     </row>
@@ -2756,12 +2756,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>339 (67)</t>
+          <t>353 (66)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>570 (69)</t>
+          <t>587 (69)</t>
         </is>
       </c>
     </row>
@@ -2773,72 +2773,72 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>30 (5.9)</t>
+          <t>31 (5.8)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>52 (6.3)</t>
+          <t>55 (6.5)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
+          <t>1.10</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>0.65, 1.85</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>0.712</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>1.21</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>0.70, 2.08</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>0.484</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>0.60, 1.90</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>0.814</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
           <t>1.15</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>0.67, 1.96</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>0.608</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>1.28</t>
-        </is>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>0.73, 2.24</t>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>0.381</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>1.14</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>0.62, 2.05</t>
-        </is>
-      </c>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>0.673</t>
-        </is>
-      </c>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>1.25</t>
-        </is>
-      </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>0.67, 2.29</t>
+          <t>0.63, 2.08</t>
         </is>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>0.481</t>
+          <t>0.639</t>
         </is>
       </c>
     </row>
@@ -2850,12 +2850,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>91 (18)</t>
+          <t>98 (18)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>158 (19)</t>
+          <t>162 (19)</t>
         </is>
       </c>
     </row>
@@ -2874,12 +2874,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>101 (20)</t>
+          <t>110 (21)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>185 (22)</t>
+          <t>193 (23)</t>
         </is>
       </c>
     </row>
@@ -2891,57 +2891,57 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>100 (20)</t>
+          <t>102 (19)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>170 (21)</t>
+          <t>172 (20)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>1.02</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>0.73, 1.54</t>
+          <t>0.71, 1.48</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>0.769</t>
+          <t>0.909</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>0.97</t>
+          <t>0.93</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>0.65, 1.44</t>
+          <t>0.64, 1.37</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>0.879</t>
+          <t>0.725</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>0.89</t>
+          <t>0.88</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>0.59, 1.34</t>
+          <t>0.59, 1.33</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>0.572</t>
+          <t>0.551</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -2951,12 +2951,12 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>0.52, 1.24</t>
+          <t>0.53, 1.22</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>0.332</t>
+          <t>0.312</t>
         </is>
       </c>
     </row>
@@ -2968,72 +2968,72 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>304 (60)</t>
+          <t>318 (60)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>467 (56)</t>
+          <t>482 (57)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.08</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>0.83, 1.54</t>
+          <t>0.80, 1.46</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>0.448</t>
+          <t>0.627</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>1.04</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>0.75, 1.43</t>
+          <t>0.74, 1.37</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>0.825</t>
+          <t>0.973</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.08</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>0.79, 1.56</t>
+          <t>0.78, 1.50</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>0.549</t>
+          <t>0.658</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>0.99</t>
+          <t>0.98</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>0.69, 1.41</t>
+          <t>0.70, 1.37</t>
         </is>
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>0.945</t>
+          <t>0.893</t>
         </is>
       </c>
     </row>
@@ -3045,7 +3045,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>4 (0.8)</t>
+          <t>4 (0.7)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3069,12 +3069,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>112 (22)</t>
+          <t>118 (22)</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>177 (21)</t>
+          <t>183 (21)</t>
         </is>
       </c>
     </row>
@@ -3086,57 +3086,57 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>125 (25)</t>
+          <t>131 (25)</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>231 (28)</t>
+          <t>236 (28)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>0.81</t>
+          <t>0.82</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>0.57, 1.16</t>
+          <t>0.59, 1.16</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>0.252</t>
+          <t>0.270</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
+          <t>0.84</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>0.59, 1.19</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>0.329</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
           <t>0.85</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>0.59, 1.23</t>
-        </is>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>0.396</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
-        <is>
-          <t>0.83</t>
-        </is>
-      </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>0.56, 1.21</t>
+          <t>0.58, 1.24</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>0.331</t>
+          <t>0.406</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -3146,12 +3146,12 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>0.59, 1.30</t>
+          <t>0.60, 1.29</t>
         </is>
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>0.515</t>
+          <t>0.507</t>
         </is>
       </c>
     </row>
@@ -3163,72 +3163,72 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>129 (25)</t>
+          <t>139 (26)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>199 (24)</t>
+          <t>206 (24)</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>0.68, 1.36</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>0.820</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>0.68, 1.40</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>0.891</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
           <t>0.91</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>0.64, 1.31</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>0.627</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>0.93</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>0.64, 1.35</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>0.713</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>0.88</t>
-        </is>
-      </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>0.59, 1.30</t>
+          <t>0.62, 1.33</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>0.511</t>
+          <t>0.613</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>0.87</t>
+          <t>0.89</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>0.58, 1.30</t>
+          <t>0.60, 1.32</t>
         </is>
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>0.495</t>
+          <t>0.577</t>
         </is>
       </c>
     </row>
@@ -3240,72 +3240,72 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>88 (17)</t>
+          <t>89 (17)</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>133 (16)</t>
+          <t>137 (16)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>0.91</t>
+          <t>0.87</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>0.61, 1.36</t>
+          <t>0.59, 1.28</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>0.648</t>
+          <t>0.470</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>0.94</t>
+          <t>0.89</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>0.62, 1.41</t>
+          <t>0.59, 1.33</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>0.755</t>
+          <t>0.567</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>1.04</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>0.67, 1.61</t>
+          <t>0.65, 1.53</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>0.870</t>
+          <t>0.992</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>1.02</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>0.67, 1.66</t>
+          <t>0.66, 1.59</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>0.815</t>
+          <t>0.924</t>
         </is>
       </c>
     </row>
@@ -3317,12 +3317,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>55 (11)</t>
+          <t>57 (11)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>87 (11)</t>
+          <t>90 (11)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3332,42 +3332,42 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>0.55, 1.37</t>
+          <t>0.56, 1.36</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>0.553</t>
+          <t>0.543</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>0.94</t>
+          <t>0.92</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>0.58, 1.50</t>
+          <t>0.58, 1.46</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>0.788</t>
+          <t>0.733</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>0.81</t>
+          <t>0.83</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>0.49, 1.34</t>
+          <t>0.50, 1.35</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>0.420</t>
+          <t>0.455</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
@@ -3377,12 +3377,12 @@
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>0.51, 1.44</t>
+          <t>0.52, 1.43</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>0.571</t>
+          <t>0.563</t>
         </is>
       </c>
     </row>
@@ -3401,12 +3401,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>304 (60)</t>
+          <t>321 (60)</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>492 (59)</t>
+          <t>508 (60)</t>
         </is>
       </c>
     </row>
@@ -3418,12 +3418,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>178 (35)</t>
+          <t>187 (35)</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>280 (34)</t>
+          <t>287 (34)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3433,57 +3433,57 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>0.85, 1.45</t>
+          <t>0.86, 1.44</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>0.428</t>
+          <t>0.414</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.17</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>0.89, 1.55</t>
+          <t>0.89, 1.53</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>0.243</t>
+          <t>0.255</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>1.02</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>0.76, 1.35</t>
+          <t>0.77, 1.36</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>0.938</t>
+          <t>0.865</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>0.81, 1.48</t>
+          <t>0.82, 1.47</t>
         </is>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>0.561</t>
+          <t>0.540</t>
         </is>
       </c>
     </row>
@@ -3495,72 +3495,72 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>27 (5.3)</t>
+          <t>26 (4.9)</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>53 (6.4)</t>
+          <t>55 (6.5)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>0.71</t>
+          <t>0.64</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>0.41, 1.20</t>
+          <t>0.37, 1.09</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>0.204</t>
+          <t>0.106</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>0.74</t>
+          <t>0.66</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>0.42, 1.29</t>
+          <t>0.37, 1.14</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>0.296</t>
+          <t>0.144</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>0.57</t>
+          <t>0.53</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>0.31, 1.02</t>
+          <t>0.29, 0.95</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>0.064</t>
+          <t>0.035</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>0.61</t>
+          <t>0.55</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>0.32, 1.11</t>
+          <t>0.29, 1.01</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>0.110</t>
+          <t>0.057</t>
         </is>
       </c>
     </row>
@@ -3596,12 +3596,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>55 (11)</t>
+          <t>63 (12)</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>206 (25)</t>
+          <t>209 (25)</t>
         </is>
       </c>
     </row>
@@ -3613,42 +3613,42 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>82 (16)</t>
+          <t>85 (16)</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>171 (21)</t>
+          <t>176 (21)</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>1.70</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>1.10, 2.63</t>
+          <t>0.98, 2.27</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>0.018</t>
+          <t>0.063</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>1.78</t>
+          <t>1.51</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>1.10, 2.89</t>
+          <t>0.95, 2.40</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>0.018</t>
+          <t>0.079</t>
         </is>
       </c>
     </row>
@@ -3660,42 +3660,42 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>81 (16)</t>
+          <t>84 (16)</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>166 (20)</t>
+          <t>170 (20)</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>2.02</t>
+          <t>1.79</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>1.30, 3.16</t>
+          <t>1.17, 2.75</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>0.002</t>
+          <t>0.007</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>2.04</t>
+          <t>1.74</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
         <is>
-          <t>1.25, 3.36</t>
+          <t>1.08, 2.80</t>
         </is>
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>0.005</t>
+          <t>0.023</t>
         </is>
       </c>
     </row>
@@ -3707,22 +3707,22 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>100 (20)</t>
+          <t>103 (19)</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>151 (18)</t>
+          <t>159 (19)</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>2.89</t>
+          <t>2.40</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1.81, 4.64</t>
+          <t>1.53, 3.78</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -3732,12 +3732,12 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>3.14</t>
+          <t>2.51</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>1.87, 5.30</t>
+          <t>1.53, 4.16</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
@@ -3754,12 +3754,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>191 (38)</t>
+          <t>199 (37)</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>133 (16)</t>
+          <t>138 (16)</t>
         </is>
       </c>
     </row>
@@ -3778,12 +3778,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>26 (5.1)</t>
+          <t>29 (5.4)</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>164 (20)</t>
+          <t>168 (20)</t>
         </is>
       </c>
     </row>
@@ -3795,42 +3795,42 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>483 (95)</t>
+          <t>505 (95)</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>663 (80)</t>
+          <t>684 (80)</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>1.64</t>
+          <t>1.33</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>0.79, 3.44</t>
+          <t>0.65, 2.73</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>0.188</t>
+          <t>0.440</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>1.89</t>
+          <t>1.52</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>0.88, 4.11</t>
+          <t>0.72, 3.23</t>
         </is>
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>0.103</t>
+          <t>0.271</t>
         </is>
       </c>
     </row>
@@ -3849,12 +3849,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>60 (12)</t>
+          <t>61 (11)</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>172 (21)</t>
+          <t>180 (21)</t>
         </is>
       </c>
     </row>
@@ -3866,42 +3866,42 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>228 (45)</t>
+          <t>236 (44)</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>342 (41)</t>
+          <t>350 (41)</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>1.38</t>
+          <t>1.46</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>0.93, 2.08</t>
+          <t>0.99, 2.18</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>0.113</t>
+          <t>0.060</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>1.40</t>
+          <t>1.46</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>0.92, 2.13</t>
+          <t>0.97, 2.20</t>
         </is>
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>0.117</t>
+          <t>0.072</t>
         </is>
       </c>
     </row>
@@ -3913,22 +3913,22 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>183 (36)</t>
+          <t>194 (36)</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>141 (17)</t>
+          <t>146 (17)</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>2.49</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>1.42, 3.66</t>
+          <t>1.57, 3.98</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
@@ -3938,12 +3938,12 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>2.43</t>
+          <t>2.66</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>1.49, 3.99</t>
+          <t>1.65, 4.32</t>
         </is>
       </c>
       <c r="O88" t="inlineStr">
@@ -3960,12 +3960,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>38 (7.5)</t>
+          <t>43 (8.1)</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>172 (21)</t>
+          <t>176 (21)</t>
         </is>
       </c>
     </row>
@@ -3984,12 +3984,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>378 (74)</t>
+          <t>389 (73)</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>504 (61)</t>
+          <t>520 (61)</t>
         </is>
       </c>
     </row>
@@ -4001,42 +4001,42 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>65 (13)</t>
+          <t>71 (13)</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>83 (10)</t>
+          <t>85 (10.0)</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>0.93</t>
+          <t>0.99</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>0.59, 1.44</t>
+          <t>0.64, 1.53</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>0.741</t>
+          <t>0.959</t>
         </is>
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>0.91</t>
+          <t>0.98</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>0.57, 1.43</t>
+          <t>0.62, 1.53</t>
         </is>
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>0.670</t>
+          <t>0.916</t>
         </is>
       </c>
     </row>
@@ -4048,42 +4048,42 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>15 (2.9)</t>
+          <t>16 (3.0)</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>32 (3.9)</t>
+          <t>34 (4.0)</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>0.76</t>
+          <t>0.73</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>0.35, 1.58</t>
+          <t>0.34, 1.47</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>0.473</t>
+          <t>0.385</t>
         </is>
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>0.65</t>
+          <t>0.58</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>0.30, 1.38</t>
+          <t>0.27, 1.21</t>
         </is>
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>0.273</t>
+          <t>0.156</t>
         </is>
       </c>
     </row>
@@ -4095,42 +4095,42 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>25 (4.9)</t>
+          <t>29 (5.4)</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>44 (5.3)</t>
+          <t>45 (5.3)</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>0.55, 2.00</t>
+          <t>0.66, 2.27</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>0.852</t>
+          <t>0.498</t>
         </is>
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>1.03</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>0.53, 1.96</t>
+          <t>0.61, 2.11</t>
         </is>
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>0.938</t>
+          <t>0.674</t>
         </is>
       </c>
     </row>
@@ -4142,12 +4142,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>26 (5.1)</t>
+          <t>29 (5.4)</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>164 (20)</t>
+          <t>168 (20)</t>
         </is>
       </c>
     </row>
@@ -4166,12 +4166,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>203 (40)</t>
+          <t>211 (40)</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>419 (51)</t>
+          <t>435 (51)</t>
         </is>
       </c>
     </row>
@@ -4183,22 +4183,22 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>173 (34)</t>
+          <t>177 (33)</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>146 (18)</t>
+          <t>147 (17)</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>2.13</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>1.51, 2.95</t>
+          <t>1.54, 2.97</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -4208,12 +4208,12 @@
       </c>
       <c r="M98" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>2.15</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>1.50, 2.99</t>
+          <t>1.53, 3.01</t>
         </is>
       </c>
       <c r="O98" t="inlineStr">
@@ -4230,12 +4230,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>133 (26)</t>
+          <t>146 (27)</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>262 (32)</t>
+          <t>270 (32)</t>
         </is>
       </c>
     </row>
@@ -4254,12 +4254,12 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>237 (47)</t>
+          <t>242 (45)</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>480 (58)</t>
+          <t>497 (58)</t>
         </is>
       </c>
     </row>
@@ -4271,12 +4271,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>153 (30)</t>
+          <t>159 (30)</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>106 (13)</t>
+          <t>109 (13)</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -4286,7 +4286,7 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>1.57, 3.19</t>
+          <t>1.58, 3.16</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -4301,7 +4301,7 @@
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>1.56, 3.25</t>
+          <t>1.58, 3.23</t>
         </is>
       </c>
       <c r="O102" t="inlineStr">
@@ -4318,7 +4318,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>21 (4.1)</t>
+          <t>22 (4.1)</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -4328,32 +4328,32 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>4.07</t>
+          <t>4.15</t>
         </is>
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>1.60, 11.0</t>
+          <t>1.66, 11.1</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>0.004</t>
+          <t>0.003</t>
         </is>
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>3.96</t>
+          <t>3.97</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
         <is>
-          <t>1.53, 10.9</t>
+          <t>1.55, 10.9</t>
         </is>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>0.006</t>
+          <t>0.005</t>
         </is>
       </c>
     </row>
@@ -4365,12 +4365,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>98 (19)</t>
+          <t>111 (21)</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>232 (28)</t>
+          <t>237 (28)</t>
         </is>
       </c>
     </row>
@@ -4389,12 +4389,12 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>364 (72)</t>
+          <t>377 (71)</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>584 (71)</t>
+          <t>602 (71)</t>
         </is>
       </c>
     </row>
@@ -4406,42 +4406,42 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>94 (18)</t>
+          <t>99 (19)</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>66 (8.0)</t>
+          <t>70 (8.2)</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>1.77</t>
+          <t>1.76</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>1.06, 2.97</t>
+          <t>1.07, 2.92</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>0.031</t>
+          <t>0.027</t>
         </is>
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>1.79</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t>1.05, 3.07</t>
+          <t>1.04, 2.95</t>
         </is>
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>0.034</t>
+          <t>0.035</t>
         </is>
       </c>
     </row>
@@ -4453,12 +4453,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>51 (10)</t>
+          <t>58 (11)</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>177 (21)</t>
+          <t>180 (21)</t>
         </is>
       </c>
     </row>
@@ -4477,12 +4477,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>188 (37)</t>
+          <t>196 (37)</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>288 (35)</t>
+          <t>295 (35)</t>
         </is>
       </c>
     </row>
@@ -4494,42 +4494,42 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>122 (24)</t>
+          <t>127 (24)</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>111 (13)</t>
+          <t>116 (14)</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>0.95</t>
+          <t>0.89</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>0.59, 1.51</t>
+          <t>0.56, 1.40</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>0.824</t>
+          <t>0.611</t>
         </is>
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>0.88</t>
+          <t>0.83</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
         <is>
-          <t>0.54, 1.41</t>
+          <t>0.52, 1.33</t>
         </is>
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>0.586</t>
+          <t>0.439</t>
         </is>
       </c>
     </row>
@@ -4541,12 +4541,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>199 (39)</t>
+          <t>211 (40)</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>428 (52)</t>
+          <t>441 (52)</t>
         </is>
       </c>
     </row>
@@ -4565,12 +4565,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>73 (14)</t>
+          <t>74 (14)</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>68 (8.2)</t>
+          <t>70 (8.2)</t>
         </is>
       </c>
     </row>
@@ -4582,42 +4582,42 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>366 (72)</t>
+          <t>380 (71)</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>517 (63)</t>
+          <t>534 (63)</t>
         </is>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>1.28</t>
+          <t>1.38</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>0.81, 2.03</t>
+          <t>0.88, 2.16</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>0.282</t>
+          <t>0.162</t>
         </is>
       </c>
       <c r="M115" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.22</t>
         </is>
       </c>
       <c r="N115" t="inlineStr">
         <is>
-          <t>0.70, 1.82</t>
+          <t>0.77, 1.96</t>
         </is>
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>0.624</t>
+          <t>0.398</t>
         </is>
       </c>
     </row>
@@ -4629,12 +4629,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>70 (14)</t>
+          <t>80 (15)</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>242 (29)</t>
+          <t>248 (29)</t>
         </is>
       </c>
     </row>

</xml_diff>